<commit_message>
feat(orders): Rasmiy qabul buyruqlari (T-40/1, T-40/2) kiritildi, talaba kartasida ko'rsatildi va davomat jurnali to'liq yangilandi
</commit_message>
<xml_diff>
--- a/hisobotlar/Davomat_Jurnali_Uchun_Malumotlar.xlsx
+++ b/hisobotlar/Davomat_Jurnali_Uchun_Malumotlar.xlsx
@@ -689,7 +689,7 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K6" s="8" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="J7" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K7" s="13" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K8" s="8" t="inlineStr">
@@ -835,7 +835,7 @@
       </c>
       <c r="J9" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K9" s="13" t="inlineStr">
@@ -885,7 +885,7 @@
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K10" s="8" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="J11" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K11" s="13" t="inlineStr">
@@ -985,7 +985,7 @@
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K12" s="8" t="inlineStr">
@@ -1035,7 +1035,7 @@
       </c>
       <c r="J13" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K13" s="13" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K14" s="8" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="J15" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K15" s="13" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K16" s="8" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="J17" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K17" s="13" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K18" s="8" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="J19" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K19" s="13" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K20" s="8" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="J21" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K21" s="13" t="inlineStr">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K22" s="8" t="inlineStr">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="J23" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K23" s="13" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K24" s="8" t="inlineStr">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="J25" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K25" s="13" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K26" s="8" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="J27" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K27" s="13" t="inlineStr">
@@ -1745,7 +1745,7 @@
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K28" s="8" t="inlineStr">
@@ -1795,7 +1795,7 @@
       </c>
       <c r="J29" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K29" s="13" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K30" s="8" t="inlineStr">
@@ -1895,7 +1895,7 @@
       </c>
       <c r="J31" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K31" s="13" t="inlineStr">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="J32" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K32" s="8" t="inlineStr">
@@ -1991,7 +1991,7 @@
       </c>
       <c r="J33" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K33" s="13" t="inlineStr">
@@ -2041,7 +2041,7 @@
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K34" s="8" t="inlineStr">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="J35" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K35" s="13" t="inlineStr">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K36" s="8" t="inlineStr">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="J37" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K37" s="13" t="inlineStr">
@@ -2241,7 +2241,7 @@
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K38" s="8" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="J39" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
       <c r="K39" s="13" t="inlineStr">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/1 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5176,7 +5176,7 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/1 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5201,7 +5201,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/1 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5226,7 +5226,7 @@
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/1 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5251,7 +5251,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/1 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5276,7 +5276,7 @@
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/1 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5301,7 +5301,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/1 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5326,7 +5326,7 @@
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/1 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5351,7 +5351,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/1 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5376,7 +5376,7 @@
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/1 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5401,7 +5401,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/1 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5426,7 +5426,7 @@
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/1 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5451,7 +5451,7 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/1 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5476,7 +5476,7 @@
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/1 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5501,7 +5501,7 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5526,7 +5526,7 @@
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5551,7 +5551,7 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5576,7 +5576,7 @@
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5601,7 +5601,7 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5626,7 +5626,7 @@
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5651,7 +5651,7 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5676,7 +5676,7 @@
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5701,7 +5701,7 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5726,7 +5726,7 @@
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5751,7 +5751,7 @@
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5776,7 +5776,7 @@
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5801,7 +5801,7 @@
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       <c r="E34" s="4" t="inlineStr"/>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5872,7 +5872,7 @@
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5897,7 +5897,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5922,7 +5922,7 @@
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5943,7 +5943,7 @@
       <c r="E38" s="4" t="inlineStr"/>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5968,7 +5968,7 @@
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -5993,7 +5993,7 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6018,7 +6018,7 @@
       </c>
       <c r="F41" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6039,7 +6039,7 @@
       <c r="E42" s="4" t="inlineStr"/>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6064,7 +6064,7 @@
       </c>
       <c r="F43" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6089,7 +6089,7 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6114,7 +6114,7 @@
       </c>
       <c r="F45" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6139,7 +6139,7 @@
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6164,7 +6164,7 @@
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6189,7 +6189,7 @@
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6214,7 +6214,7 @@
       </c>
       <c r="F49" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6239,7 +6239,7 @@
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6264,7 +6264,7 @@
       </c>
       <c r="F51" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6289,7 +6289,7 @@
       </c>
       <c r="F52" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6314,7 +6314,7 @@
       </c>
       <c r="F53" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6335,7 +6335,7 @@
       <c r="E54" s="4" t="inlineStr"/>
       <c r="F54" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6360,7 +6360,7 @@
       </c>
       <c r="F55" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6385,7 +6385,7 @@
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6410,7 +6410,7 @@
       </c>
       <c r="F57" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6460,7 +6460,7 @@
       </c>
       <c r="F59" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6485,7 +6485,7 @@
       </c>
       <c r="F60" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6510,7 +6510,7 @@
       </c>
       <c r="F61" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6535,7 +6535,7 @@
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6556,7 +6556,7 @@
       <c r="E63" s="9" t="inlineStr"/>
       <c r="F63" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6577,7 +6577,7 @@
       <c r="E64" s="4" t="inlineStr"/>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6602,7 +6602,7 @@
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6627,7 +6627,7 @@
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6652,7 +6652,7 @@
       </c>
       <c r="F67" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6677,7 +6677,7 @@
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6702,7 +6702,7 @@
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6727,7 +6727,7 @@
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6752,7 +6752,7 @@
       </c>
       <c r="F71" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6773,7 +6773,7 @@
       <c r="E72" s="4" t="inlineStr"/>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6798,7 +6798,7 @@
       </c>
       <c r="F73" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6823,7 +6823,7 @@
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6848,7 +6848,7 @@
       </c>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6873,7 +6873,7 @@
       </c>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6898,7 +6898,7 @@
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6923,7 +6923,7 @@
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6948,7 +6948,7 @@
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6973,7 +6973,7 @@
       </c>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -6998,7 +6998,7 @@
       </c>
       <c r="F81" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="F82" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7048,7 +7048,7 @@
       </c>
       <c r="F83" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7073,7 +7073,7 @@
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7098,7 +7098,7 @@
       </c>
       <c r="F85" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7123,7 +7123,7 @@
       </c>
       <c r="F86" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7148,7 +7148,7 @@
       </c>
       <c r="F87" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7173,7 +7173,7 @@
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7198,7 +7198,7 @@
       </c>
       <c r="F89" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7223,7 +7223,7 @@
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7248,7 +7248,7 @@
       </c>
       <c r="F91" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7273,7 +7273,7 @@
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7298,7 +7298,7 @@
       </c>
       <c r="F93" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7323,7 +7323,7 @@
       </c>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7348,7 +7348,7 @@
       </c>
       <c r="F95" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7373,7 +7373,7 @@
       </c>
       <c r="F96" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7398,7 +7398,7 @@
       </c>
       <c r="F97" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7423,7 +7423,7 @@
       </c>
       <c r="F98" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7448,7 +7448,7 @@
       </c>
       <c r="F99" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7473,7 +7473,7 @@
       </c>
       <c r="F100" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7498,7 +7498,7 @@
       </c>
       <c r="F101" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7523,7 +7523,7 @@
       </c>
       <c r="F102" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7548,7 +7548,7 @@
       </c>
       <c r="F103" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7573,7 +7573,7 @@
       </c>
       <c r="F104" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7598,7 +7598,7 @@
       </c>
       <c r="F105" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7619,7 +7619,7 @@
       <c r="E106" s="4" t="inlineStr"/>
       <c r="F106" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7644,7 +7644,7 @@
       </c>
       <c r="F107" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7669,7 +7669,7 @@
       </c>
       <c r="F108" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7694,7 +7694,7 @@
       </c>
       <c r="F109" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7719,7 +7719,7 @@
       </c>
       <c r="F110" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7744,7 +7744,7 @@
       </c>
       <c r="F111" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7769,7 +7769,7 @@
       </c>
       <c r="F112" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7794,7 +7794,7 @@
       </c>
       <c r="F113" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7819,7 +7819,7 @@
       </c>
       <c r="F114" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7844,7 +7844,7 @@
       </c>
       <c r="F115" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7869,7 +7869,7 @@
       </c>
       <c r="F116" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7894,7 +7894,7 @@
       </c>
       <c r="F117" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7919,7 +7919,7 @@
       </c>
       <c r="F118" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7944,7 +7944,7 @@
       </c>
       <c r="F119" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7969,7 +7969,7 @@
       </c>
       <c r="F120" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -7994,7 +7994,7 @@
       </c>
       <c r="F121" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8019,7 +8019,7 @@
       </c>
       <c r="F122" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8044,7 +8044,7 @@
       </c>
       <c r="F123" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8069,7 +8069,7 @@
       </c>
       <c r="F124" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8094,7 +8094,7 @@
       </c>
       <c r="F125" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8119,7 +8119,7 @@
       </c>
       <c r="F126" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8144,7 +8144,7 @@
       </c>
       <c r="F127" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8169,7 +8169,7 @@
       </c>
       <c r="F128" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8194,7 +8194,7 @@
       </c>
       <c r="F129" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8219,7 +8219,7 @@
       </c>
       <c r="F130" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8244,7 +8244,7 @@
       </c>
       <c r="F131" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8269,7 +8269,7 @@
       </c>
       <c r="F132" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8294,7 +8294,7 @@
       </c>
       <c r="F133" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8319,7 +8319,7 @@
       </c>
       <c r="F134" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="F135" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8369,7 +8369,7 @@
       </c>
       <c r="F136" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8394,7 +8394,7 @@
       </c>
       <c r="F137" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8419,7 +8419,7 @@
       </c>
       <c r="F138" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8444,7 +8444,7 @@
       </c>
       <c r="F139" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8469,7 +8469,7 @@
       </c>
       <c r="F140" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8490,7 +8490,7 @@
       <c r="E141" s="9" t="inlineStr"/>
       <c r="F141" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8515,7 +8515,7 @@
       </c>
       <c r="F142" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8540,7 +8540,7 @@
       </c>
       <c r="F143" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8565,7 +8565,7 @@
       </c>
       <c r="F144" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8590,7 +8590,7 @@
       </c>
       <c r="F145" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8615,7 +8615,7 @@
       </c>
       <c r="F146" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8640,7 +8640,7 @@
       </c>
       <c r="F147" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8665,7 +8665,7 @@
       </c>
       <c r="F148" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8690,7 +8690,7 @@
       </c>
       <c r="F149" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8715,7 +8715,7 @@
       </c>
       <c r="F150" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8740,7 +8740,7 @@
       </c>
       <c r="F151" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8765,7 +8765,7 @@
       </c>
       <c r="F152" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8790,7 +8790,7 @@
       </c>
       <c r="F153" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8815,7 +8815,7 @@
       </c>
       <c r="F154" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8840,7 +8840,7 @@
       </c>
       <c r="F155" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8865,7 +8865,7 @@
       </c>
       <c r="F156" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8890,7 +8890,7 @@
       </c>
       <c r="F157" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8911,7 +8911,7 @@
       <c r="E158" s="4" t="inlineStr"/>
       <c r="F158" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8936,7 +8936,7 @@
       </c>
       <c r="F159" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8961,7 +8961,7 @@
       </c>
       <c r="F160" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -8986,7 +8986,7 @@
       </c>
       <c r="F161" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9011,7 +9011,7 @@
       </c>
       <c r="F162" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9036,7 +9036,7 @@
       </c>
       <c r="F163" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9061,7 +9061,7 @@
       </c>
       <c r="F164" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9086,7 +9086,7 @@
       </c>
       <c r="F165" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9111,7 +9111,7 @@
       </c>
       <c r="F166" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9136,7 +9136,7 @@
       </c>
       <c r="F167" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9161,7 +9161,7 @@
       </c>
       <c r="F168" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9186,7 +9186,7 @@
       </c>
       <c r="F169" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9207,7 +9207,7 @@
       <c r="E170" s="4" t="inlineStr"/>
       <c r="F170" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9228,7 +9228,7 @@
       <c r="E171" s="9" t="inlineStr"/>
       <c r="F171" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9253,7 +9253,7 @@
       </c>
       <c r="F172" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9278,7 +9278,7 @@
       </c>
       <c r="F173" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9303,7 +9303,7 @@
       </c>
       <c r="F174" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9328,7 +9328,7 @@
       </c>
       <c r="F175" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9353,7 +9353,7 @@
       </c>
       <c r="F176" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9378,7 +9378,7 @@
       </c>
       <c r="F177" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9403,7 +9403,7 @@
       </c>
       <c r="F178" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9424,7 +9424,7 @@
       <c r="E179" s="9" t="inlineStr"/>
       <c r="F179" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9449,7 +9449,7 @@
       </c>
       <c r="F180" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9474,7 +9474,7 @@
       </c>
       <c r="F181" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9499,7 +9499,7 @@
       </c>
       <c r="F182" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9524,7 +9524,7 @@
       </c>
       <c r="F183" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9549,7 +9549,7 @@
       </c>
       <c r="F184" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9574,7 +9574,7 @@
       </c>
       <c r="F185" s="9" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>
@@ -9599,7 +9599,7 @@
       </c>
       <c r="F186" s="4" t="inlineStr">
         <is>
-          <t>№ 18, 04.09.2025</t>
+          <t>T-40/2 02.09.2026</t>
         </is>
       </c>
     </row>

</xml_diff>